<commit_message>
Refactor life insurance agent portal to enforce sequential business flow and add missing proposal & payment screens
</commit_message>
<xml_diff>
--- a/betacare_agent_portal_fsd.xlsx
+++ b/betacare_agent_portal_fsd.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Agent Registration" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Agent Login" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Agent Dashboard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lead Management" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="New Lead Form" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Quote Generation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Policies &amp; Underwriting" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Settings &amp; Config" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Registration" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Login" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Dashboard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Management" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Lead Form" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quote Generation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policies &amp; Underwriting" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings &amp; Config" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,17 +459,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
     <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -563,7 +563,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Returns user back to previous page in onboarding wizard</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Navigates user to login page</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Validates and submits agent onboarding data to backend registration API</t>
         </is>
       </c>
     </row>
@@ -699,12 +699,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Must be checked</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Required declaration check for regulatory compliance</t>
         </is>
       </c>
     </row>
@@ -736,22 +736,22 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Email validation format regex</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Primary contact and notification address for agency registration alerts</t>
         </is>
       </c>
     </row>
@@ -783,22 +783,22 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>File</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 5MB</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>PDF/JPG/PNG format only</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bank details proof required for commission payout setups</t>
         </is>
       </c>
     </row>
@@ -830,22 +830,22 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>File</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 5MB</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>PDF/JPG/PNG format only</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Identity and address verification KYC document</t>
         </is>
       </c>
     </row>
@@ -877,22 +877,22 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>File</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 5MB</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>PDF/JPG/PNG format only</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tax identification verification KYC document</t>
         </is>
       </c>
     </row>
@@ -924,22 +924,22 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>12-digit length check</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Identity proof matches official Aadhaar registration data</t>
         </is>
       </c>
     </row>
@@ -971,22 +971,22 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Min 9, Max 18</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric digits only</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bank account number for commission payouts</t>
         </is>
       </c>
     </row>
@@ -1018,22 +1018,22 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10-digit format</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Primary number for OTP setups and communication</t>
         </is>
       </c>
     </row>
@@ -1065,22 +1065,22 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10-digit format</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Secondary emergency contact number</t>
         </is>
       </c>
     </row>
@@ -1112,22 +1112,22 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Min 10, Max 12</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric digits only</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alternative telephone number for agent records</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1159,22 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>6-digit length</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Address verification check for sales region mapping</t>
         </is>
       </c>
     </row>
@@ -1206,22 +1206,22 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 2</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Must be positive number</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>IRDAI compliance criteria verification for sales licensing</t>
         </is>
       </c>
     </row>
@@ -1253,22 +1253,22 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Must match Bank Account holder name exactly</t>
         </is>
       </c>
     </row>
@@ -1300,22 +1300,22 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 50</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Select from Independent / Corporate</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sets corporate commission sharing profiles</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 15</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Unique ID assigned to the agent in database records</t>
         </is>
       </c>
     </row>
@@ -1394,22 +1394,22 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bank name for routing payouts</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bank branch location for payout routing</t>
         </is>
       </c>
     </row>
@@ -1488,22 +1488,22 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 50</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>City location for territorial sales mapping</t>
         </is>
       </c>
     </row>
@@ -1535,12 +1535,12 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Registered entity name for corporate agency structures</t>
         </is>
       </c>
     </row>
@@ -1582,22 +1582,22 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Regulatory requirement tracking for conflict of interest</t>
         </is>
       </c>
     </row>
@@ -1629,22 +1629,22 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Checks minimum education eligibility for insurance advisors</t>
         </is>
       </c>
     </row>
@@ -1676,22 +1676,22 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>11-digit alphanumeric format check</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>IFSC validation mapping against RBI bank list</t>
         </is>
       </c>
     </row>
@@ -1723,12 +1723,12 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 20</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Verifies active licensing status with national regulator</t>
         </is>
       </c>
     </row>
@@ -1770,22 +1770,22 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Legal name matching identity proof</t>
         </is>
       </c>
     </row>
@@ -1817,22 +1817,22 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 50</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Required checking for foreign/domestic broker classifications</t>
         </is>
       </c>
     </row>
@@ -1864,22 +1864,22 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Designated nominee for commission inheritance</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>PAN format regex check (5 alpha, 4 numeric, 1 alpha)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Required tax registration validation</t>
         </is>
       </c>
     </row>
@@ -1958,22 +1958,22 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Preferred territory alignment for lead routing allocations</t>
         </is>
       </c>
     </row>
@@ -2005,22 +2005,22 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic characters only</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Historical agency registry alignment checks</t>
         </is>
       </c>
     </row>
@@ -2052,12 +2052,12 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Primary insurance product lines advisor wishes to sell</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphabetic</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Demographic tracking for sales routing</t>
         </is>
       </c>
     </row>
@@ -2162,6 +2162,53 @@
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>User device native biometric authentication</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>0. Create Account (Agent Registration)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Onboarding Progress Bar</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Visual Component</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Step Tracker Grid</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Displays active wizard stage (1: Document KYC, 2: Personal, 3: Professional, 4: Bank Details)</t>
         </is>
       </c>
     </row>
@@ -2176,11 +2223,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
@@ -2270,7 +2317,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -2433,7 +2480,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Login (Navigation)</t>
+          <t>LOGIN TERMINAL Button</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2468,7 +2515,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Submits request to backend auth endpoint</t>
+          <t>Submits request to backend auth endpoint POST /auth/login</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2562,289 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Redirects user to password reset path</t>
+          <t>Redirects user to forgot password modal overlay page</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reset Password Email Input</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Max 100</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Email validation</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Input to receive password reset OTP request</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Send OTP Button</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Triggers OTP dispatch request via SMS/Email and shows OTP input</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>OTP Code Input</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Numeric (6-digit)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>6-digit match</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>OTP code input block matching sent challenge</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>New Password Input</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Masked Input</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Min 8, Max 50</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Must have uppercase, lowercase, number</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Sets new password parameter in system records</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Confirm New Password Input</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Masked Input</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Min 8, Max 50</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Must match New Password</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Verifies password entry precision</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1. Agent Login Portal</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Submit Password Reset Button</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Submits password updates to database, resetting user credential logs</t>
         </is>
       </c>
     </row>
@@ -2530,13 +2859,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -2740,27 +3069,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Register a New Lead</t>
+          <t>Leads Assigned Counter</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Card Widget</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Clickable UI Element</t>
+          <t>Numeric Counter</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Non-Mandatory</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -2775,7 +3104,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Directly routes the agent to the 6-stage Lead intake wizard</t>
+          <t>Displays total leads currently assigned to the Agent ID</t>
         </is>
       </c>
     </row>
@@ -2787,27 +3116,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Live Activity Timeline</t>
+          <t>Register a New Lead</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>List Panel</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Chronological Log Feed</t>
+          <t>Clickable UI Element</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Non-Mandatory</t>
+          <t>Mandatory</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Alphanumeric</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -2822,7 +3151,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Queries and displays the latest 5 actions made in the DB</t>
+          <t>Directly routes the agent to the 6-stage Lead intake wizard</t>
         </is>
       </c>
     </row>
@@ -2834,42 +3163,371 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Sidebar Navigation Link Rows</t>
+          <t>Premium Collections Dashboard Chart</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>Chart Panel</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>SVG Interactive Bar Chart</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Renders graphical metrics mapping Q1, Q2, Q3, Q4 collections</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Premium Metric Tooltip</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Tooltip Widget</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Hover Text (₹)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Displays exact Indian Rupee amount details on bar hover</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Live Activity Timeline Feed</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>List Panel</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Chronological Log Feed</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Queries and displays the latest 5 actions made in the DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Timeline Log Entry</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Visual Row</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Text String with Status Bullet</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Color-coded status row tracking policy issuances, underwrite updates, or lead creations</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Sidebar Navigation Branding Block</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Brand Component</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>White Container Block + Logo</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Displays BetaCare Life Shield Brand logo block</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Sidebar Navigation Links</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
           <t>Menu Panel</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>List of Links</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Provides central access links to Dashboard, Leads, Underwriting, Policies, and Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Agent Profile Footer Card</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>User Card Widget</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Rounded initials avatar + profile link</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Circular avatar displaying broker name 'aditi' and link to Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2. Agent Dashboard</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Exit Session (Logout)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Action Link</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Clickable link</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Destroys active session JWT token and redirects user to Agent Login Portal</t>
         </is>
       </c>
     </row>
@@ -2884,13 +3542,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -3047,7 +3705,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Leads Data Grid</t>
+          <t>Leads Data Grid Table</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -3094,17 +3752,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>View Details Action</t>
+          <t>Lead Tracking ID Link</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Link</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Clickable UI Element</t>
+          <t>Clickable Hashtag ID</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3114,12 +3772,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -3129,7 +3787,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Loads detailed Lead profile page workspace</t>
+          <t>Loads detailed Lead profile page details workspace (e.g. #06318E)</t>
         </is>
       </c>
     </row>
@@ -3177,6 +3835,288 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Bypasses to quote calculation options using existing lead metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>KPI statistics: Total Leads</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Card Widget</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Numeric Counter</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Displays sum of all captured leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>KPI statistics: Hot Leads</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Card Widget</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Numeric Counter</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Displays count of high-intent leads (orange badges)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>KPI statistics: Warm Leads</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Card Widget</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Numeric Counter</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Displays count of moderate-intent leads (yellow badges)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>KPI statistics: Cold Leads</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Card Widget</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Numeric Counter</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Displays count of low-intent leads (blue badges)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>KPI statistics: Quotations</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Card Widget</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Numeric Counter</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Displays count of actively shared quotations files</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>3. Lead Management</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Understanding Lead Temperature Panel</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Panel Block</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Text Description Rows</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Static instructional card detailing the definition of Hot, Warm, Cold lead segmentations</t>
         </is>
       </c>
     </row>
@@ -3191,13 +4131,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -3260,7 +4200,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>Full Legal Name</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -3354,17 +4294,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Email Address</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Dropdown</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>name@domain.com</t>
+          <t>Selection List</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -3374,7 +4314,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Alphanumeric</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3384,12 +4324,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Valid email structure regex match</t>
+          <t>Select from Male / Female / Other</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Enforces unique constraint checks in Lead records</t>
+          <t>Input used in actuarial underwriting estimations</t>
         </is>
       </c>
     </row>
@@ -3401,17 +4341,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Mobile No.</t>
+          <t>Email Address</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>10-digit Numeric</t>
+          <t>name@domain.com</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3421,22 +4361,22 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Numeric</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Max 100</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>10-digit length check</t>
+          <t>Valid email structure regex match</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Standard phone validation checks for customer contacts</t>
+          <t>Enforces unique constraint checks in Lead records</t>
         </is>
       </c>
     </row>
@@ -3448,7 +4388,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Annual Income</t>
+          <t>Mobile No.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -3458,7 +4398,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>10-digit Numeric</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3473,17 +4413,17 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Max 12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Must be greater than 0</t>
+          <t>10-digit length check</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Alters underwriting risk categorization</t>
+          <t>Standard phone validation checks for customer contacts</t>
         </is>
       </c>
     </row>
@@ -3495,17 +4435,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Plan Type</t>
+          <t>Annual Income</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Dropdown</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Selection List</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3515,22 +4455,22 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 12</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Select from Term / Whole Life / ULIP</t>
+          <t>Must be greater than 0</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Sets calculation formulas for quotation estimation</t>
+          <t>Alters underwriting risk categorization</t>
         </is>
       </c>
     </row>
@@ -3542,17 +4482,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Sum Assured Amount</t>
+          <t>Plan Type</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>Dropdown</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Selection List</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3562,22 +4502,22 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Numeric</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Max 12</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Must meet minimum sum limits per plan</t>
+          <t>Select from Term / Whole Life / ULIP</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Core underwriting metric for automated decisions</t>
+          <t>Sets calculation formulas for quotation estimation</t>
         </is>
       </c>
     </row>
@@ -3589,17 +4529,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Premium Payment Frequency</t>
+          <t>Sum Assured Target</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Dropdown</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Selection List</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3609,22 +4549,22 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Numeric</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 12</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Select from Monthly / Quarterly / Annual</t>
+          <t>Must meet minimum sum limits per plan</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Adjusts base premium math breakdown dynamically</t>
+          <t>Core underwriting metric for automated decisions</t>
         </is>
       </c>
     </row>
@@ -3636,17 +4576,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Upload Aadhaar File</t>
+          <t>Premium Payment Frequency</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Dropdown</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>PDF/JPG/PNG</t>
+          <t>Selection List</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3656,22 +4596,22 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Max 5MB</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>File extension must be PDF/JPG/PNG</t>
+          <t>Select from Monthly / Quarterly / Annual</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Critical KYC document criteria required by IRDAI regulations</t>
+          <t>Adjusts base premium math breakdown dynamically</t>
         </is>
       </c>
     </row>
@@ -3683,7 +4623,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Upload PAN File</t>
+          <t>Upload Aadhaar File</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -3730,17 +4670,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>KYC Declaration Check</t>
+          <t>Upload PAN File</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>File Upload</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Y/N</t>
+          <t>PDF/JPG/PNG</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -3750,22 +4690,22 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>File</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 5MB</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Must be checked</t>
+          <t>File extension must be PDF/JPG/PNG</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Locks data submission until compliance verification is confirmed</t>
+          <t>Critical KYC document criteria required by IRDAI regulations</t>
         </is>
       </c>
     </row>
@@ -3777,42 +4717,559 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Submit Profile</t>
+          <t>KYC Declaration Checkbox</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Y/N</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Must be checked</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Locks data submission until compliance verification is confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Submit Profile Button</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
           <t>Button</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Clickable UI Element</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Sends lead details to backend Rules Engine for automated screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Lead Details: Profile Context Banner</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Header Component</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Title Panel</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Context panel displaying Name, Unique Database ID, and HOT/WARM badge</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Quick Communication: Call CTA</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Phone action button</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Triggers softphone interface call to prospect number</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Quick Communication: WhatsApp CTA</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Chat action button</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Opens whatsapp web client prefilled with contact message</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Quick Communication: Email CTA</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Mail action button</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Launches client default mail composer prefilled with email address</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Underwriting Health Score Metric</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Visual Card</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Gauge Score (x/100)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Calculated lead health assessment metrics scoring index</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AI Policy &amp; Upsell Advisor Panel</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Container Block</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Card Panel Panel</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Renders dynamic agent output suggestions block</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AI Advice Suitability Badge</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Badge Widget</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Color-coded Pill Label</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Optimal Fit, Moderate Fit, Low Fit rating</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Visual rating output returned by sales_lead_advisor CrewAI execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>AI Dynamic Pitch Notes</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Text Area</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Bulleted Markdown list</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Detailed selling guidance and objections refutations returned by QA test architect and analyst agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Re-Analyze Profile Button</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Manually re-triggers backend execution of Sales Lead Advisor Agent crew to update advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>4. New Lead Form Wizard</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>AI Agent progress loader</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Loader Widget</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Visual spinner</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Indicates status of background Agentic run when re-analyzing lead profile data</t>
         </is>
       </c>
     </row>
@@ -3827,17 +5284,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
     <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -3906,7 +5363,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Currency Format</t>
+          <t>Currency Format (₹)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -3953,7 +5410,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Currency Format</t>
+          <t>Currency Format (₹)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -4000,7 +5457,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Currency Format</t>
+          <t>Currency Format (₹)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -4084,7 +5541,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Confirm Plan Selection</t>
+          <t>Confirm Plan Selection Button</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -4120,6 +5577,194 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Saves plan choice configuration details to lead state profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5. Quote Generation</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Download Proposal PDF Button</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Generates detailed PDF illustration and saves copy locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5. Quote Generation</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Compare Plans Matrix Button</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Launches comparison overlay comparing premiums across standard products</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>5. Quote Generation</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Fulfillment review terms checkbox</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Y/N</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Must be checked</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Confirms that customer has agreed to proposal parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>5. Quote Generation</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Submit Proposal Button</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Submits the finalized proposal to the manual Underwriting Review Queue</t>
         </is>
       </c>
     </row>
@@ -4134,17 +5779,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
     <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -4203,7 +5848,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Underwriting Case Queue Grid</t>
+          <t>Underwriting Case Queue Data Grid</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -4250,27 +5895,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Risk Category Badge</t>
+          <t>Trigger Underwriting Agent Button</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Badge</t>
+          <t>Button</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Color-coded Label</t>
+          <t>Clickable UI Element</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Non-Mandatory</t>
+          <t>Mandatory</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -4285,7 +5930,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Visual category indicator: Low (Green), Medium (Yellow), High (Red)</t>
+          <t>Triggers manual execution of the Underwriting Risk Assessment Agent crew</t>
         </is>
       </c>
     </row>
@@ -4297,32 +5942,32 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Notes &amp; Comments Entry Box</t>
+          <t>Underwriting Risk Agent feedback card</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Textarea</t>
+          <t>Container Block</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>String Paragraph</t>
+          <t>Card Panel Panel</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Non-Mandatory</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Alphanumeric</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Max 500</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4332,7 +5977,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Permits underwriters to document audit findings</t>
+          <t>Wrapper widget presenting the AI underwriter findings</t>
         </is>
       </c>
     </row>
@@ -4344,27 +5989,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Approve Application</t>
+          <t>AI Risk Rating Badge</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Badge</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Clickable UI Element</t>
+          <t>Color-coded Label</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Non-Mandatory</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -4374,12 +6019,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Low (Green), Medium (Yellow), High (Red) risk rating</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Transitions lead state to Issued, creating a dynamic active policy record</t>
+          <t>Computed risk tier returned by underwrite_agent.py execution</t>
         </is>
       </c>
     </row>
@@ -4391,32 +6036,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Reject Application</t>
+          <t>AI Actuary Notes Textbox</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Textarea</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Clickable UI Element</t>
+          <t>String Paragraph</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Non-Mandatory</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Alphanumeric</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Max 1000</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -4426,7 +6071,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Rejects the case and records the stated rejection notes in timeline logs</t>
+          <t>Contains detailed, professional justification notes returned by compliance officer agent</t>
         </is>
       </c>
     </row>
@@ -4438,42 +6083,230 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>Approve Application</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Transitions lead state to Issued, creating a dynamic active policy record</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6. Underwriting &amp; Policies</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reject Application</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Clickable UI Element</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Rejects the case and records the stated rejection notes in timeline logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>6. Underwriting &amp; Policies</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Rejection Reason Notes Field</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Textarea</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>String Paragraph</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Non-Mandatory</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Max 500</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Permits manual input justification notes for case rejection</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>6. Underwriting &amp; Policies</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
           <t>Active Policies List Grid</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>List Grid</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Non-Mandatory</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Displays active policies detailing Policy Number, Sum Assured, Premium, Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>6. Underwriting &amp; Policies</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Policy Number Link</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Clickable Alphanumeric ID</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Max 20</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Loads policy details workspace showing transaction lists and certificate downloads</t>
         </is>
       </c>
     </row>
@@ -4488,11 +6321,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
@@ -4698,7 +6531,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Save Changes Settings</t>
+          <t>Save Changes Settings Button</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -4734,6 +6567,53 @@
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Commits setting updates to local storage state and remote database profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>7. Settings Page</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Agent API Configuration Logs</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Textarea</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>System log entries</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Alphanumeric</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Displays real-time logs indicating API response codes, database check status, and token expiry alerts</t>
         </is>
       </c>
     </row>

</xml_diff>